<commit_message>
Update QA report after retest
</commit_message>
<xml_diff>
--- a/docs/Dataset_Quality_Checker_QA_Test_Cases.xlsx
+++ b/docs/Dataset_Quality_Checker_QA_Test_Cases.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="528">
   <si>
     <t xml:space="preserve">Dataset Quality Checker — QA Test Cases</t>
   </si>
@@ -1019,6 +1019,9 @@
     <t xml:space="preserve">Uploading 03_header_only.csv displayed the red error “The file has no data rows.” and no report was generated. But The error message “The file has no data rows” remained visible after moving to the next dataset.</t>
   </si>
   <si>
+    <t xml:space="preserve">Failed first run (B-001); passed retest on live site 12 Oct 2026 after fix.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-050</t>
   </si>
   <si>
@@ -1333,7 +1336,7 @@
     <t xml:space="preserve">Binary file renamed to .csv was rejected with the expected red error message; no report was generated. BUT The error “This looks like a binary file (for example an image or an Excel file renamed to .csv), not a text CSV file.” remained visible after moving to the next dataset.</t>
   </si>
   <si>
-    <t xml:space="preserve">Stale binary-file validation error persists after selecting a new dataset.</t>
+    <t xml:space="preserve">Failed first run (B-002); passed retest on live site 12 Oct 2026 after fix.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-067</t>
@@ -1403,7 +1406,7 @@
     <t xml:space="preserve">Opening the application in Opera, Microsoft Edge, and Firefox displayed “Method Not Allowed.” The application could not be tested in those browsers.</t>
   </si>
   <si>
-    <t xml:space="preserve">Reproduced in Opera, Edge, and Firefox.</t>
+    <t xml:space="preserve">Failed first run because the URL tested was /dqc/analyze (B-003, now fixed). Rerun in Opera, Edge and Firefox using https://saabz.pythonanywhere.com/dqc/ still pending.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-071</t>
@@ -1475,10 +1478,10 @@
     <t xml:space="preserve">The previous “The file has no data rows” error remains visible after moving to the next dataset.</t>
   </si>
   <si>
-    <t xml:space="preserve">Retest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed 12 Oct 2026 (commit 119d52d). Retest pending.</t>
+    <t xml:space="preserve">Fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed in commit 1c1ae25. Retested on live site 12 Oct 2026: error clears when a new file is chosen; 05_one_row.csv report loads (score 85).</t>
   </si>
   <si>
     <t xml:space="preserve">B-002</t>
@@ -1499,6 +1502,9 @@
     <t xml:space="preserve">The previous binary-file error remains visible after selecting the next dataset.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fixed in commit 1c1ae25. Retested on live site 12 Oct 2026: binary-file error clears when a new file is chosen; clean file report loads.</t>
+  </si>
+  <si>
     <t xml:space="preserve">B-003</t>
   </si>
   <si>
@@ -1515,6 +1521,9 @@
   </si>
   <si>
     <t xml:space="preserve">Opera, Microsoft Edge, and Firefox display “Method Not Allowed,” preventing further testing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed in commit 1c1ae25. Cause: /dqc/analyze opened directly (the URL shown after a check) returned 405 in every browser. Now redirects to the upload page; retested on live site 12 Oct 2026 (Chromium).</t>
   </si>
   <si>
     <t xml:space="preserve">File (in qa_test_data.zip)</t>
@@ -2135,9 +2144,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>1789920</xdr:colOff>
+      <xdr:colOff>1789560</xdr:colOff>
       <xdr:row>49</xdr:row>
-      <xdr:rowOff>772560</xdr:rowOff>
+      <xdr:rowOff>772200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2151,7 +2160,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="16758360" y="21879000"/>
-          <a:ext cx="1736640" cy="772560"/>
+          <a:ext cx="1736280" cy="772200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2177,9 +2186,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>10800</xdr:colOff>
+      <xdr:colOff>10440</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>867960</xdr:rowOff>
+      <xdr:rowOff>867600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2193,7 +2202,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12462480" y="419040"/>
-          <a:ext cx="1786320" cy="810720"/>
+          <a:ext cx="1785960" cy="810360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2214,9 +2223,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>6480</xdr:colOff>
+      <xdr:colOff>6120</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>757440</xdr:rowOff>
+      <xdr:rowOff>757080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2230,7 +2239,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12466080" y="1291320"/>
-          <a:ext cx="1778400" cy="742320"/>
+          <a:ext cx="1778040" cy="741960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2251,9 +2260,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1816920</xdr:colOff>
+      <xdr:colOff>1816560</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>761400</xdr:rowOff>
+      <xdr:rowOff>761040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2267,7 +2276,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12462480" y="2103120"/>
-          <a:ext cx="1759680" cy="715680"/>
+          <a:ext cx="1759320" cy="715320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2832,11 +2841,11 @@
       </c>
       <c r="D10" s="11" t="n">
         <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$73,$B10,'Test Cases'!$H$2:$H$73,"Pass")</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E10" s="11" t="n">
         <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$73,$B10,'Test Cases'!$H$2:$H$73,"Fail")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" s="11" t="n">
         <f aca="false">COUNTIFS('Test Cases'!$B$2:$B$73,$B10,'Test Cases'!$H$2:$H$73,"Blocked")</f>
@@ -2848,7 +2857,7 @@
       </c>
       <c r="H10" s="12" t="n">
         <f aca="false">IFERROR(D10/(C10-G10),0)</f>
-        <v>0.894736842105263</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2890,11 +2899,11 @@
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">SUM(D6:D11)</f>
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E12" s="13" t="n">
         <f aca="false">SUM(E6:E11)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="13" t="n">
         <f aca="false">SUM(F6:F11)</f>
@@ -2906,7 +2915,7 @@
       </c>
       <c r="H12" s="14" t="n">
         <f aca="false">IFERROR(D12/(C12-G12),0)</f>
-        <v>0.958333333333333</v>
+        <v>0.986111111111111</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2934,7 +2943,7 @@
       </c>
       <c r="C18" s="11" t="n">
         <f aca="false">COUNTIFS('Bug Log'!$E$3:$E$199,B18,'Bug Log'!$H$3:$H$199,"&lt;&gt;Fixed",'Bug Log'!$H$3:$H$199,"&lt;&gt;Closed")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4481,154 +4490,154 @@
         <v>322</v>
       </c>
       <c r="H50" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I50" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="J50" s="20"/>
+        <v>26</v>
+      </c>
+      <c r="I50" s="20"/>
+      <c r="J50" s="20" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="17" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B51" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D51" s="19" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G51" s="20" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="H51" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I51" s="20"/>
       <c r="J51" s="20" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="17" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B52" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D52" s="19" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E52" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G52" s="20" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="H52" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I52" s="20"/>
       <c r="J52" s="20" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B53" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C53" s="19" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D53" s="19" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E53" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G53" s="20" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H53" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I53" s="20"/>
       <c r="J53" s="20" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B54" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D54" s="19" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E54" s="19" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F54" s="19" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G54" s="20" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="H54" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I54" s="20"/>
       <c r="J54" s="20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B55" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D55" s="19" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E55" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G55" s="20" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H55" s="20" t="s">
         <v>26</v>
@@ -4640,25 +4649,25 @@
     </row>
     <row r="56" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="17" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B56" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D56" s="19" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E56" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F56" s="19" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G56" s="20" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H56" s="20" t="s">
         <v>26</v>
@@ -4670,55 +4679,55 @@
     </row>
     <row r="57" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="17" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B57" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E57" s="19" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F57" s="19" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G57" s="20" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H57" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I57" s="20"/>
       <c r="J57" s="20" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="17" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B58" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D58" s="19" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E58" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F58" s="19" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G58" s="20" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H58" s="20" t="s">
         <v>26</v>
@@ -4730,327 +4739,325 @@
     </row>
     <row r="59" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="17" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B59" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D59" s="19" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E59" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F59" s="19" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G59" s="20" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="H59" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I59" s="20"/>
       <c r="J59" s="20" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="17" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B60" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E60" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F60" s="19" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G60" s="20" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H60" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I60" s="20"/>
       <c r="J60" s="20" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="17" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B61" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F61" s="19" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G61" s="20" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="H61" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I61" s="20"/>
       <c r="J61" s="20" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="17" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B62" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F62" s="19" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G62" s="20" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="H62" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I62" s="20"/>
       <c r="J62" s="20" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="17" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B63" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D63" s="19" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F63" s="19" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G63" s="20" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="H63" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I63" s="20"/>
       <c r="J63" s="20" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B64" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C64" s="19" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E64" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F64" s="19" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G64" s="20" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H64" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I64" s="20"/>
       <c r="J64" s="20" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="17" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B65" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D65" s="19" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F65" s="19" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G65" s="20" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="H65" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I65" s="20"/>
       <c r="J65" s="20" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="17" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B66" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E66" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F66" s="19" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G66" s="20" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="H66" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I66" s="20"/>
       <c r="J66" s="20" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="17" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B67" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C67" s="19" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D67" s="19" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E67" s="19" t="s">
         <v>245</v>
       </c>
       <c r="F67" s="19" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G67" s="20" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="H67" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="I67" s="20" t="s">
-        <v>54</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="I67" s="20"/>
       <c r="J67" s="20" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="17" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B68" s="18" t="s">
         <v>49</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D68" s="19" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E68" s="19" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F68" s="19" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G68" s="20" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H68" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I68" s="20"/>
       <c r="J68" s="20" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="17" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B69" s="18" t="s">
         <v>50</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D69" s="19" t="s">
         <v>70</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F69" s="19" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="G69" s="20" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="H69" s="20" t="s">
         <v>26</v>
@@ -5062,25 +5069,25 @@
     </row>
     <row r="70" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="17" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B70" s="18" t="s">
         <v>50</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D70" s="19" t="s">
         <v>177</v>
       </c>
       <c r="E70" s="19" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F70" s="19" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G70" s="20" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="H70" s="20" t="s">
         <v>26</v>
@@ -5092,25 +5099,25 @@
     </row>
     <row r="71" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="17" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B71" s="18" t="s">
         <v>50</v>
       </c>
       <c r="C71" s="19" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D71" s="19" t="s">
         <v>81</v>
       </c>
       <c r="E71" s="19" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F71" s="19" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G71" s="20" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="H71" s="20" t="s">
         <v>41</v>
@@ -5119,30 +5126,30 @@
         <v>54</v>
       </c>
       <c r="J71" s="20" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="17" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B72" s="18" t="s">
         <v>50</v>
       </c>
       <c r="C72" s="19" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D72" s="19" t="s">
         <v>81</v>
       </c>
       <c r="E72" s="19" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F72" s="19" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G72" s="20" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="H72" s="20" t="s">
         <v>26</v>
@@ -5154,25 +5161,25 @@
     </row>
     <row r="73" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="17" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B73" s="18" t="s">
         <v>50</v>
       </c>
       <c r="C73" s="19" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D73" s="19" t="s">
         <v>177</v>
       </c>
       <c r="E73" s="19" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F73" s="19" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G73" s="20" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H73" s="20" t="s">
         <v>26</v>
@@ -5236,123 +5243,123 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>23</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>12</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B3" s="20" t="s">
         <v>318</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E3" s="20" t="s">
         <v>54</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I3" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E4" s="20" t="s">
         <v>54</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E5" s="20" t="s">
         <v>54</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5975,10 +5982,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5986,15 +5993,15 @@
         <v>81</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6002,7 +6009,7 @@
         <v>320</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6010,39 +6017,39 @@
         <v>133</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="25" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6050,7 +6057,7 @@
         <v>139</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6058,15 +6065,15 @@
         <v>145</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6074,79 +6081,79 @@
         <v>151</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="25" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="25" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="25" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="25" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="25" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="25" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="25" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6154,15 +6161,15 @@
         <v>116</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="25" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6170,7 +6177,7 @@
         <v>126</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
     </row>
   </sheetData>

</xml_diff>